<commit_message>
limpiezas-planeadas.xlsx sale de un script, y documenta lo de Sensores
El Excel se editaba a mano. Ahora su contenido vive en
tools/limpiezas/datos.py (una celda por linea, legible en un diff) y
generar.py lo arma con el formato de siempre. Regenerado contra el
original: mismo contenido, negritas, colores y anchos; solo cambian 48
celdas de renglones que se habian agregado sin formato, que ahora quedan
ajustadas como las demas.

Nuevo: las limpiezas 19-22 (SERIE SENSOR de los 22 sensores en BAJA, las
2 series sin sensor, SENSOR reducido a SI/NO TIENE con sus 39 cambios, y
3 columnas con dueno por decidir), por que no se tocan TIPO DE
COMBUSTIBLE ni RAZON SOCIAL, la suposicion de un sensor por vehiculo, y
como se midio en produccion.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/limpiezas-planeadas.xlsx
+++ b/limpiezas-planeadas.xlsx
@@ -31,17 +31,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
@@ -70,6 +67,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C6E0B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2E2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
@@ -78,18 +85,8 @@
         <fgColor rgb="00FF9999"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6E0B4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2E2E2"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -97,47 +94,37 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -505,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -754,7 +741,7 @@
           <t>Una columna sin nombre usable, y el error se arrastra a cualquier copia del libro.</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>HECHO</t>
         </is>
@@ -834,7 +821,7 @@
           <t>Tres hojas huérfanas del padre. No se puede saber qué línea se reactivó ni qué equipo se desechó sin cruzar a mano.</t>
         </is>
       </c>
-      <c r="H8" s="12" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>YA NO APLICA</t>
         </is>
@@ -914,7 +901,7 @@
           <t>Una columna que promete un dato y nunca lo da.</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>DECISION DE NEGOCIO</t>
         </is>
@@ -1074,7 +1061,7 @@
           <t>Dos fondos activos de $10,000 cada uno a nombre de personas que ya no trabajan aquí. De todo lo que salió hoy, esto es lo más urgente.</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>URGENTE</t>
         </is>
@@ -1281,6 +1268,166 @@
       <c r="H19" s="3" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>VEHICULOS</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Vaciar SERIE SENSOR de los 22 vehículos cuyo sensor está en BAJA</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>22 celdas</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Al dar de baja un sensor nadie limpiaba VEHICULOS. Medido en producción el 01/10/2026: los 22 son reales (los mismos en el libro del equipo), no datos de prueba. Decisión de Ayrton (01/10/2026): al dar de baja, se vacía. Desde ahora INSTALACION DE SENSORES es la dueña de SERIE SENSOR y SENSOR en VEHICULOS (al revés de las demás columnas, donde VEHICULOS es la dueña).</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>VEHICULOS sigue mostrando como instalada la serie de un sensor que ya se retiró.</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>VEHICULOS</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Vaciar SERIE SENSOR de CTA0295 y CTA0481: tienen serie pero ningún renglón de sensor</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>2 celdas</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Sus series (G95Z0ZTP77A1 y G9W5HX33RZ6H) no aparecen en INSTALACION DE SENSORES. CAVEAT: puede ser un sensor instalado que nunca se registró. Si es así, lo correcto es DAR DE ALTA el sensor, no borrar la serie. Revisarlos antes de sincronizar: la pantalla de Relaciones los lista uno por uno.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Una serie que no se puede rastrear a ninguna instalación ni responsiva.</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>VEHICULOS</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Reducir SENSOR a dos valores: SI TIENE SENSOR / NO TIENE SENSOR</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>39 celdas</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Decisión de Ayrton (01/10/2026). Se calcula del sensor: ACTIVO → SI TIENE; en BAJA o sin renglón → NO TIENE. Pasan a NO TIENE 36: CANCELADO 18, SENSOR TI 5, NO COMPATIBLE 2, NO APLICA AUTO DG 2, EN PROCESO DE INSTALACION 1, vacío 2, y 6 que dicen SI TIENE sin sensor activo. Pasan a SI TIENE 3 con sensor activo (CANCELADO 2, SENSOR TI 1). CAVEAT: se PIERDE el matiz de CANCELADO, NO COMPATIBLE, SENSOR TI, etc. — si hace falta, tendrá que vivir en otra columna. Y los 6 "SI TIENE" sin activo pueden ser sensores no registrados, igual que la limpieza #20.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>SENSOR dice una cosa y la hoja de sensores otra en 39 vehículos, y nadie sabe cuál creer.</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>VEHICULOS / HOLOGRAMAS / INSPECCION VEHICULAR</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Medir y decidir el dueño de 3 columnas que se llaman igual en VEHICULOS y en una hija</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>3 columnas</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Aparecieron al revisar Sensores y NO están en el mapa de Relaciones: HOLOGRAMAS.NO ECONOMICO (no se sabe quién manda), INSPECCION VEHICULAR.POLIZA SEGURO (probablemente la póliza del día: bitácora) y VEHICULOS.VERIFICACION (SI / NO) (huele a resumen de VERIFICACIONES, como SENSOR).</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Pueden estar desincronizadas sin que nada lo detecte, igual que SERIE SENSOR hasta hoy.</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>RE-MEDIR</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1653,6 +1800,60 @@
       <c r="E13" s="2" t="inlineStr">
         <is>
           <t>4 de 145</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>INSTALACION DE SENSORES.TIPO DE COMBUSTIBLE y HOLOGRAMAS.RAZON SOCIAL</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Se llaman igual que una columna de VEHICULOS, así que parecen copias desincronizadas</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Significan otra cosa. En Sensores es el PRODUCTO que carga la unidad (MAGNA/PREMIUM/DIESEL) y en VEHICULOS el tipo de motor (GASOLINA/DIESEL); en Hologramas es la empresa del contrato de la tarjeta, no la dueña del vehículo. Por eso NO están en el mapa de Relaciones y nunca se sincronizan.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2 columnas</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>INSTALACION DE SENSORES → VEHICULOS: un solo renglón de sensor por vehículo</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Una sincronización "simple" podría tener que escoger entre varios sensores de la misma unidad</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Hoy no hace falta escoger: en producción cada vehículo tiene a lo más un renglón de sensor (208 de 208). Es una SUPOSICIÓN medida, no una regla del sistema: si algún día una unidad tiene dos renglones (una reinstalación), la sincronización lo reporta como llave repetida y NO toca VEHICULOS hasta que alguien lo resuelva.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>208 de 208</t>
         </is>
       </c>
     </row>
@@ -1856,7 +2057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1876,7 +2077,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
@@ -1888,7 +2089,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Libro</t>
         </is>
@@ -1900,7 +2101,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
@@ -1912,7 +2113,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Método</t>
         </is>
@@ -1924,7 +2125,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Ojo con las lecturas truncadas</t>
         </is>
@@ -1936,7 +2137,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Documentos relacionados</t>
         </is>
@@ -1948,7 +2149,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Lo que NO se midió</t>
         </is>
@@ -1960,7 +2161,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Estado de Líneas</t>
         </is>
@@ -1971,51 +2172,63 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Lo que NO se midió (actualizado)</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Ya se midieron las dos cosas que faltaban de Caja Chica: los datos de persona contra COLABORADORES y la aritmética de los arqueos. Queda pendiente de Líneas la distribución de los cambios en el tiempo.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="46" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Un límite que hay que saber</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>ARQUEOS no tiene fórmulas: sus totales son valores literales que escribió AppSheet. Eso NO impide verificarlos —cuadran los 145— pero sí significa que la fórmula vive en AppSheet y no en el spreadsheet. La que aplica la confirmó Ayrton el 30/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="52" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Una corrección de este archivo</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>La primera versión reportó una brecha de $986,185.11 en TOTAL GENERAL. Estaba mal: sumé 11 de las 12 columnas de la fórmula y omití DISPONIBLE CUENTA BANCARIA, que suma exactamente esa cantidad. ARQUEOS cuadra al centavo en los 145 arqueos. Queda anotado para que nadie persiga un problema que no existe.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="62" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Lineas se reestructuro el 30/09/2026</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Hubo junta del area y los cambios ya estan en el libro COMPARTIDO del equipo (1fC77Uu1...), no en produccion. Se eliminaron 4 pestañas: HISTORIAL_REASIGNACIONES, REACTIVACION DE LINEAS, SOLICITUD DE LINEAS y BITACORA DE DESECHO. Por eso las limpiezas 5, 7, 4 y 8 cambiaron de estado. Verificado despues de la reestructuracion: NUCO sigue siendo llave unica, 1,615 de 1,615. Detalle en docs/lineas-homologacion.md, en el aviso de arriba.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Sensores ↔ VEHICULOS (01/10/2026)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Medido en PRODUCCIÓN (1h5ibDsmVtrG27rwMaOvj-lm08QZUHzDv3woPmkfRQrk), solo lectura. Producción no tiene la columna ID, así que ahí se emparejó por SERIE VEHICULO, igual que Relaciones.gs. Resultado: 648 vehículos y 208 renglones de sensor (186 ACTIVO, 22 BAJA), con a lo más UN renglón por vehículo (208 de 208). En el libro del equipo salen además 3 casos que son datos de prueba y no existen en producción: la serie 'prueba', AUT0025 con dos sensores activos y una serie activa en otro vehículo.</t>
         </is>
       </c>
     </row>
@@ -2241,41 +2454,53 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="46" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Cómo se emparejó</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>CAJAS CHICAS no tiene número de empleado. Se emparejó por CORREO ELECTRONICO DE RESPONSABLE (216 de 285, 76%) y por nombre (277, 97%); con cualquiera de las dos, 283 de 285 (99%).</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Lo bueno</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>El 99% de las cajas encuentran a su responsable en el catálogo. Es la tasa más alta de las tres familias: en Líneas es 45%.</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="46" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Lo que NO se debe sincronizar</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>PUESTO (17%), SEDE (26%) y OFICINA (28%). Que SEDE dé exactamente el mismo 26% que en Líneas refuerza que esa columna significa algo distinto del catálogo de personas.</t>
         </is>
       </c>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2319,7 +2544,7 @@
           <t>Las columnas M 0,50 … B 1000,00: ¿piezas o importes?</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>PIEZAS, 145 de 145</t>
         </is>
@@ -2336,7 +2561,7 @@
           <t>TOTAL M = suma de monedas × denominación</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>145 de 145</t>
         </is>
@@ -2353,7 +2578,7 @@
           <t>TOTAL B = suma de billetes × denominación</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>145 de 145</t>
         </is>
@@ -2370,7 +2595,7 @@
           <t>TOTAL EFECTIVO = TOTAL M + TOTAL B</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>145 de 145</t>
         </is>
@@ -2387,7 +2612,7 @@
           <t>TOTAL GENERAL = la suma de sus 12 partes</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>145 de 145  ✓</t>
         </is>
@@ -2404,7 +2629,7 @@
           <t>DIFERENCIA = TOTAL GENERAL − MONTO CAJA</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>144 de 145</t>
         </is>
@@ -2421,7 +2646,7 @@
           <t>Arqueos sin efectivo físico (TOTAL EFECTIVO = 0)</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>109 de 145</t>
         </is>
@@ -2433,55 +2658,61 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>CORRECCIÓN A UNA VERSIÓN ANTERIOR DE ESTA HOJA</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="52" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Qué decía</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Que TOTAL GENERAL no cuadraba con sus partes en 111 de 145 arqueos, con una brecha acumulada de $986,185.11 «sin explicar».</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="52" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Por qué estaba mal</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sumé 11 columnas y la fórmula tiene 12: me faltó DISPONIBLE CUENTA BANCARIA. Esa columna suma exactamente $986,185.11 — el mismo número, al centavo. La brecha era mi omisión, no un problema de los datos.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="52" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Lo que en realidad pasa</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Muchas cajas no guardan efectivo: su fondo está en una cuenta bancaria o fintech (la hoja tiene DESCRIPCION CUENTA BANCARIA y Nombre_Fintech). Por eso TOTAL EFECTIVO = 0 en 109 arqueos, y es normal.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="52" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Y sobre DIFERENCIA = 0</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>También estaba mal dicho. Con la fórmula completa, DIFERENCIA sí es un control real: compara el total de lo que hay contra el fondo autorizado. Que valga 0 significa que la caja cuadró, no que el número esté inventado.</t>
         </is>

</xml_diff>